<commit_message>
chore(curriculum): publish representation-learning — graph, /paths, audit, metrics
Flip the curriculum-graph node from "planned" to "published"; remove
from the T3 (Unsupervised & Generative) "planned" array — the track
is now feature-complete. Add two incoming edges: pca-low-rank and
shannon-entropy → representation-learning.

Re-run pnpm audit:cross-site to discharge the inbound deferred
reciprocal from formalstatistics/sufficient-statistics. Stage the
sister-side JSON diffs (formalcalculus / formalstatistics) which
reflect real cross-repo content changes captured by this audit run.

Update docs/formalml-content-metrics.xlsx with the new Topic Detail
row, refreshed Domain Summary for "unsupervised" (now 3 topics), and
a Gap Analysis "Missing code section" entry (intentional — §11.4
covers computational considerations in prose, with code living in
the executed companion notebook and the in-browser TS shared module).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalml-content-metrics.xlsx
+++ b/docs/formalml-content-metrics.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R64"/>
+  <dimension ref="A1:R65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5187,6 +5187,80 @@
       <c r="R64" t="inlineStr">
         <is>
           <t>Overview and motivation; Bayesian model selection at a glance — what RJ-MCMC computes; The trans-dimensional state space; Standard MH refresher and where it stops short; The dimension-matching auxiliary-variable construction; Reversibility of the bijection and the involution shortcut; Detailed balance with the Jacobian correction — the master acceptance ratio; The move catalog — split/merge, birth/death, and RJ-MH; Worked example A — Linear-regression variable selection (Kuo–Mallick); Worked example B — Univariate Gaussian-mixture order estimation (Richardson–Green on Galaxy data); Diagnostics for trans-dimensional chains; Computational notes; Connections and limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>unsupervised</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Representation Learning</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>7980</v>
+      </c>
+      <c r="E65" t="n">
+        <v>13</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" t="n">
+        <v>42</v>
+      </c>
+      <c r="M65" t="n">
+        <v>60</v>
+      </c>
+      <c r="N65" t="n">
+        <v>859</v>
+      </c>
+      <c r="O65" t="n">
+        <v>45</v>
+      </c>
+      <c r="P65" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>0</v>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>What is a representation, and what makes one good?; Sufficient statistics as the limit point of "good representation"; The autoencoder family; The variational autoencoder; The contrastive principle and the InfoNCE bound; SimCLR and the design space of contrastive methods; The information bottleneck perspective; Self-supervised pretext tasks beyond contrastive; Evaluating representations; Identifiability and what self-supervision cannot give you; Computational considerations; The geometry of learned representations; Connections, limits, and forward pointers</t>
         </is>
       </c>
     </row>
@@ -5716,10 +5790,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>10197.5</v>
+        <v>9458.333333333334</v>
       </c>
       <c r="D13" t="n">
         <v>6346</v>
@@ -5728,7 +5802,7 @@
         <v>14049</v>
       </c>
       <c r="F13" t="n">
-        <v>12</v>
+        <v>12.33333333333333</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -5737,7 +5811,7 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -5800,7 +5874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7159,6 +7233,33 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Representation Learning</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>unsupervised</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Missing code section</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Brief §11.4 explicitly addresses computational considerations in prose; code lives in the executed companion notebook at notebooks/representation-learning/01_representation_learning.ipynb (NumPy/SciPy for §3.2 Baldi-Hornik, §3.4 Tweedie, §5.3 InfoNCE bound, §7.2 Gaussian IB; PyTorch for §4 VAE, §5.5 contrastive trajectory, §6.2 SimCLR projection head, §12.3 neural-collapse classifier). No dedicated MDX code section by design — the in-browser TS shared module (src/components/viz/shared/representation-learning.ts) plus the four precompute scripts cover the computational surface.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(curriculum): publish bayesian-inference — metrics + brief
content-metrics.xlsx: Topic Detail row for Bayesian Inference (9991
words, 13 sections, 19 TheoremBlocks, 62 display equations, 727
inline-math spans, 30 references all with URLs). Domain Summary
recomputed for bayesian-ml (10 topics, avg 9113 words). Gap Analysis
entry for "Missing code section" (low priority — umbrella by design,
code lives in the executed companion notebook and the shared TS
module).

Handoff brief is the 1170-line pre-implementation spec — section
outlines, viz design intents, cross-site prereq verification list, and
the implementation handoff notes. Tracked here for future audit and
backport reference.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalml-content-metrics.xlsx
+++ b/docs/formalml-content-metrics.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topic Detail" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Topic Detail" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Domain Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gap Analysis" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R65"/>
+  <dimension ref="A1:R66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5261,6 +5261,80 @@
       <c r="R65" t="inlineStr">
         <is>
           <t>What is a representation, and what makes one good?; Sufficient statistics as the limit point of "good representation"; The autoencoder family; The variational autoencoder; The contrastive principle and the InfoNCE bound; SimCLR and the design space of contrastive methods; The information bottleneck perspective; Self-supervised pretext tasks beyond contrastive; Evaluating representations; Identifiability and what self-supervision cannot give you; Computational considerations; The geometry of learned representations; Connections, limits, and forward pointers</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>bayesian-ml</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Bayesian Inference</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>foundational</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>9991</v>
+      </c>
+      <c r="E66" t="n">
+        <v>13</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="n">
+        <v>19</v>
+      </c>
+      <c r="M66" t="n">
+        <v>62</v>
+      </c>
+      <c r="N66" t="n">
+        <v>727</v>
+      </c>
+      <c r="O66" t="n">
+        <v>30</v>
+      </c>
+      <c r="P66" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>0</v>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>1. Why Bayesian inference?; 2. The prior–likelihood–posterior cycle; 3. Choosing a prior; 4. Conjugate families; 5. Point estimates from a posterior; 6. The posterior predictive distribution; 7. Bayesian decision theory; 8. Sequential updating and exchangeability; 9. Hierarchical Bayes and partial pooling; 10. Bayesian model comparison; 11. Computational reality; 12. The frequentist–Bayesian dialogue; 13. Connections and limits</t>
         </is>
       </c>
     </row>
@@ -5710,10 +5784,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>9015</v>
+        <v>9113</v>
       </c>
       <c r="D11" t="n">
         <v>2764</v>
@@ -5722,7 +5796,7 @@
         <v>14873</v>
       </c>
       <c r="F11" t="n">
-        <v>9.800000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="G11" t="n">
         <v>1</v>
@@ -5731,10 +5805,10 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -5874,7 +5948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7260,6 +7334,33 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Bayesian Inference</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>bayesian-ml</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Missing code section</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Umbrella topic by design — code lives in the executed companion notebook at notebooks/bayesian-inference/01_bayesian_inference.ipynb (NumPy/SciPy/matplotlib only, no MCMC libraries). The in-browser TS shared module (src/components/viz/shared/bayesian-inference.ts) covers Beta/Normal/Bayes-factor/EB primitives for the 11 interactive viz. No dedicated MDX code section by design — the brief explicitly forward-points algorithmic content to the 13 T5 leaves.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>